<commit_message>
feat: Add health functional food ERD map and super ERD map
</commit_message>
<xml_diff>
--- a/데이터_활용사례_Playwright.xlsx
+++ b/데이터_활용사례_Playwright.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="240">
   <si>
     <t>서비스 명</t>
   </si>
@@ -172,21 +172,6 @@
   </si>
   <si>
     <t>토스(Toss)</t>
-  </si>
-  <si>
-    <t>모든 금융 계좌를 한눈에 관리하고 송금대출투자보험까지 간편하게 처리할 수 있는 올인원 핀테크 앱</t>
-  </si>
-  <si>
-    <t>건강기능식품 폐업정보
-건강기능식품판매업
-수입식품등영업신고대장
-수입식품업 폐업정보
-식육즉석판매가공업 인허가 대장
-식육즉석판매가공업 폐업정보
-식품등수입판매업정보
-식품소분업 인허가 대장
-식품소분업 폐업정보
-식품제조가공업 폐업정보 외 11종</t>
   </si>
   <si>
     <t>자사 쇼핑몰에서 식품 상품 판매자의 인허가 현황 사전 검수</t>
@@ -678,17 +663,6 @@
     <t>푸드비투비(FoodB2B)</t>
   </si>
   <si>
-    <t>건강기능식품 전문.벤처제조업인허가 현황
-건강기능식품 GMP 지정 현황
-건강기능식품판매업
-기구.용기포장제조업
-수입식품등영업신고대장
-식품등수입판매업체
-식품제조가공업정보
-식품첨가물제조업
-축산물 가공업허가정보</t>
-  </si>
-  <si>
     <t>워치독</t>
   </si>
   <si>
@@ -1135,6 +1109,35 @@
   </si>
   <si>
     <t>회수판매 중지 정보</t>
+  </si>
+  <si>
+    <t>모든 금융 계좌를 한눈에 관리하고 송금대출투자보험까지 간편하게 처리할 수 있는 올인원 핀테크 앱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>건강기능식품 폐업정보
+건강기능식품판매업
+수입식품등영업신고대장
+수입식품업 폐업정보
+식육즉석판매가공업 인허가 대장
+식육즉석판매가공업 폐업정보
+식품등수입판매업정보
+식품소분업 인허가 대장
+식품소분업 폐업정보
+식품제조가공업 폐업정보 외 11종</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>건강기능식품 전문.벤처제조업인허가 현황
+건강기능식품 GMP 지정 현황
+건강기능식품판매업
+기구.용기포장제조업
+수입식품등영업신고대장
+식품등수입판매업체
+식품제조가공업정보
+식품첨가물제조업
+축산물 가공업허가정보</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1577,7 +1580,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>10</v>
@@ -1589,7 +1592,7 @@
         <v>12</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" ht="346.5" x14ac:dyDescent="0.3">
@@ -1689,183 +1692,183 @@
         <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="F9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="2" customFormat="1" ht="165" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" ht="214.5" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="F11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" ht="198" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="F13" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" ht="231" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" ht="313.5" x14ac:dyDescent="0.3">
@@ -1873,22 +1876,22 @@
         <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
@@ -1896,7 +1899,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>9</v>
@@ -1911,7 +1914,7 @@
         <v>9</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
@@ -1919,19 +1922,19 @@
         <v>9</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
@@ -1939,19 +1942,19 @@
         <v>9</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
@@ -1959,19 +1962,19 @@
         <v>9</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20" spans="1:7" s="2" customFormat="1" ht="165" x14ac:dyDescent="0.3">
@@ -1979,19 +1982,19 @@
         <v>9</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:7" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
@@ -1999,19 +2002,19 @@
         <v>9</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:7" s="2" customFormat="1" ht="214.5" x14ac:dyDescent="0.3">
@@ -2019,19 +2022,19 @@
         <v>9</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:7" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
@@ -2039,19 +2042,19 @@
         <v>9</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:7" s="2" customFormat="1" ht="231" x14ac:dyDescent="0.3">
@@ -2059,19 +2062,19 @@
         <v>9</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="2" customFormat="1" ht="231" x14ac:dyDescent="0.3">
@@ -2079,19 +2082,19 @@
         <v>9</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="2" customFormat="1" ht="214.5" x14ac:dyDescent="0.3">
@@ -2099,19 +2102,19 @@
         <v>9</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="2" customFormat="1" ht="396" x14ac:dyDescent="0.3">
@@ -2119,19 +2122,19 @@
         <v>9</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:7" s="2" customFormat="1" ht="313.5" x14ac:dyDescent="0.3">
@@ -2139,19 +2142,19 @@
         <v>9</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="29" spans="1:7" s="2" customFormat="1" ht="231" x14ac:dyDescent="0.3">
@@ -2159,19 +2162,19 @@
         <v>9</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:7" s="2" customFormat="1" ht="165" x14ac:dyDescent="0.3">
@@ -2179,19 +2182,19 @@
         <v>9</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
@@ -2199,7 +2202,7 @@
         <v>9</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>9</v>
@@ -2211,7 +2214,7 @@
         <v>9</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="2" customFormat="1" ht="165" x14ac:dyDescent="0.3">
@@ -2219,19 +2222,19 @@
         <v>9</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="2" customFormat="1" ht="280.5" x14ac:dyDescent="0.3">
@@ -2239,19 +2242,19 @@
         <v>9</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="2" customFormat="1" ht="247.5" x14ac:dyDescent="0.3">
@@ -2259,19 +2262,19 @@
         <v>9</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="2" customFormat="1" ht="181.5" x14ac:dyDescent="0.3">
@@ -2279,19 +2282,19 @@
         <v>9</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:7" s="2" customFormat="1" ht="247.5" x14ac:dyDescent="0.3">
@@ -2299,19 +2302,19 @@
         <v>9</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:7" s="2" customFormat="1" ht="247.5" x14ac:dyDescent="0.3">
@@ -2319,19 +2322,19 @@
         <v>9</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" spans="1:7" s="2" customFormat="1" ht="165" x14ac:dyDescent="0.3">
@@ -2339,19 +2342,19 @@
         <v>9</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="39" spans="1:7" s="2" customFormat="1" ht="280.5" x14ac:dyDescent="0.3">
@@ -2359,19 +2362,19 @@
         <v>9</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="40" spans="1:7" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
@@ -2379,33 +2382,33 @@
         <v>9</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="2" customFormat="1" ht="363" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>9</v>
@@ -2414,7 +2417,7 @@
         <v>9</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="2" customFormat="1" ht="264" x14ac:dyDescent="0.3">
@@ -2422,22 +2425,22 @@
         <v>9</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="43" spans="1:7" s="2" customFormat="1" ht="264" x14ac:dyDescent="0.3">
@@ -2445,22 +2448,22 @@
         <v>9</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="F43" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
@@ -2477,13 +2480,13 @@
         <v>9</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="45" spans="1:7" s="2" customFormat="1" ht="247.5" x14ac:dyDescent="0.3">
@@ -2491,19 +2494,19 @@
         <v>9</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="46" spans="1:7" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
@@ -2511,22 +2514,22 @@
         <v>9</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="47" spans="1:7" s="2" customFormat="1" ht="330" x14ac:dyDescent="0.3">
@@ -2534,22 +2537,22 @@
         <v>9</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F47" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="G47" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="48" spans="1:7" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
@@ -2557,22 +2560,22 @@
         <v>9</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="49" spans="1:7" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
@@ -2580,36 +2583,36 @@
         <v>9</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="F49" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G49" s="2" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="50" spans="1:7" s="2" customFormat="1" ht="280.5" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>9</v>
@@ -2618,21 +2621,21 @@
         <v>9</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="51" spans="1:7" s="2" customFormat="1" ht="280.5" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>9</v>
@@ -2641,12 +2644,12 @@
         <v>9</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="52" spans="1:7" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>9</v>
@@ -2664,87 +2667,87 @@
         <v>9</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="53" spans="1:7" s="2" customFormat="1" ht="396" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>9</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="54" spans="1:7" s="2" customFormat="1" ht="363" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G54" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="55" spans="1:7" s="2" customFormat="1" ht="198" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G55" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="56" spans="1:7" s="2" customFormat="1" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>165</v>
+        <v>239</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>9</v>
@@ -2756,18 +2759,18 @@
         <v>9</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="57" spans="1:7" s="2" customFormat="1" ht="396" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>9</v>
@@ -2779,7 +2782,7 @@
         <v>9</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>